<commit_message>
feat: incluido uma nova coluna com o carimbo do revisor (A ou B)
</commit_message>
<xml_diff>
--- a/data/review/gpt-5.4-pro/step-2-review.xlsx
+++ b/data/review/gpt-5.4-pro/step-2-review.xlsx
@@ -420,13 +420,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D409"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,6 +451,11 @@
           <t>decision</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -468,6 +474,7 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -486,6 +493,7 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -504,6 +512,7 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -522,6 +531,7 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -540,6 +550,7 @@
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -558,6 +569,7 @@
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -576,6 +588,7 @@
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -594,6 +607,7 @@
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -612,6 +626,7 @@
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -630,6 +645,7 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -648,6 +664,7 @@
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -666,6 +683,7 @@
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -684,6 +702,7 @@
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -702,6 +721,7 @@
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -720,6 +740,7 @@
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -738,6 +759,7 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -756,6 +778,7 @@
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -774,6 +797,7 @@
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -792,6 +816,7 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -810,6 +835,7 @@
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -828,6 +854,7 @@
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -846,6 +873,7 @@
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -864,6 +892,7 @@
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -882,6 +911,7 @@
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -900,6 +930,7 @@
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -918,6 +949,7 @@
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -936,6 +968,7 @@
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -954,6 +987,7 @@
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -972,6 +1006,7 @@
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -990,6 +1025,7 @@
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1008,6 +1044,7 @@
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1026,6 +1063,7 @@
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1044,6 +1082,7 @@
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1062,6 +1101,7 @@
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1080,6 +1120,7 @@
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1098,6 +1139,7 @@
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1116,6 +1158,7 @@
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1134,6 +1177,7 @@
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1152,6 +1196,7 @@
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1170,6 +1215,7 @@
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1188,6 +1234,7 @@
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1206,6 +1253,7 @@
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1224,6 +1272,7 @@
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1242,6 +1291,7 @@
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1260,6 +1310,7 @@
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1278,6 +1329,7 @@
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1296,6 +1348,7 @@
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1314,6 +1367,7 @@
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1332,6 +1386,7 @@
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1350,6 +1405,7 @@
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1368,6 +1424,7 @@
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1386,6 +1443,7 @@
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1404,6 +1462,7 @@
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1422,6 +1481,7 @@
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1440,6 +1500,7 @@
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1458,6 +1519,7 @@
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1476,6 +1538,7 @@
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1494,6 +1557,7 @@
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1512,6 +1576,7 @@
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1530,6 +1595,7 @@
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1548,6 +1614,7 @@
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1566,6 +1633,7 @@
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1584,6 +1652,7 @@
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1602,6 +1671,7 @@
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1620,6 +1690,7 @@
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1638,6 +1709,7 @@
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1656,6 +1728,7 @@
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1674,6 +1747,7 @@
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1692,6 +1766,7 @@
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1710,6 +1785,7 @@
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1728,6 +1804,7 @@
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1746,6 +1823,7 @@
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1764,6 +1842,7 @@
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1782,6 +1861,7 @@
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1800,6 +1880,7 @@
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1818,6 +1899,7 @@
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1836,6 +1918,7 @@
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1854,6 +1937,7 @@
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1872,6 +1956,7 @@
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1890,6 +1975,7 @@
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1908,6 +1994,7 @@
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1926,6 +2013,7 @@
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1944,6 +2032,7 @@
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1962,6 +2051,7 @@
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1980,6 +2070,7 @@
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1998,6 +2089,7 @@
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2016,6 +2108,7 @@
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2034,6 +2127,7 @@
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2052,6 +2146,7 @@
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2070,6 +2165,7 @@
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2088,6 +2184,7 @@
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2106,6 +2203,7 @@
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2124,6 +2222,7 @@
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2142,6 +2241,7 @@
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2160,6 +2260,7 @@
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2178,6 +2279,7 @@
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2196,6 +2298,7 @@
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2214,6 +2317,7 @@
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2232,6 +2336,7 @@
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2250,6 +2355,7 @@
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2268,6 +2374,7 @@
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2286,6 +2393,7 @@
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2304,6 +2412,7 @@
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2322,6 +2431,7 @@
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2340,6 +2450,7 @@
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2358,6 +2469,7 @@
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2376,6 +2488,7 @@
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2394,6 +2507,7 @@
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2412,6 +2526,7 @@
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2430,6 +2545,7 @@
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2448,6 +2564,7 @@
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2466,6 +2583,7 @@
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2484,6 +2602,7 @@
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2502,6 +2621,7 @@
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2520,6 +2640,7 @@
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2538,6 +2659,7 @@
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2556,6 +2678,7 @@
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2574,6 +2697,7 @@
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2592,6 +2716,7 @@
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2610,6 +2735,7 @@
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2628,6 +2754,7 @@
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2646,6 +2773,7 @@
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2664,6 +2792,7 @@
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2682,6 +2811,7 @@
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2700,6 +2830,7 @@
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2718,6 +2849,7 @@
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2736,6 +2868,7 @@
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2754,6 +2887,7 @@
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2772,6 +2906,7 @@
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2790,6 +2925,7 @@
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2808,6 +2944,7 @@
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2826,6 +2963,7 @@
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2844,6 +2982,7 @@
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2862,6 +3001,7 @@
         </is>
       </c>
       <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2880,6 +3020,7 @@
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2898,6 +3039,7 @@
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2916,6 +3058,7 @@
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2934,6 +3077,7 @@
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2952,6 +3096,7 @@
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2970,6 +3115,7 @@
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2988,6 +3134,7 @@
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3006,6 +3153,7 @@
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3024,6 +3172,7 @@
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3042,6 +3191,7 @@
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3060,6 +3210,7 @@
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3078,6 +3229,7 @@
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3096,6 +3248,7 @@
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3114,6 +3267,7 @@
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3132,6 +3286,7 @@
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3150,6 +3305,7 @@
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3168,6 +3324,7 @@
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3186,6 +3343,7 @@
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3204,6 +3362,7 @@
         </is>
       </c>
       <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3222,6 +3381,7 @@
         </is>
       </c>
       <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3240,6 +3400,7 @@
         </is>
       </c>
       <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3258,6 +3419,7 @@
         </is>
       </c>
       <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3276,6 +3438,7 @@
         </is>
       </c>
       <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3294,6 +3457,7 @@
         </is>
       </c>
       <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3312,6 +3476,7 @@
         </is>
       </c>
       <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3330,6 +3495,7 @@
         </is>
       </c>
       <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3348,6 +3514,7 @@
         </is>
       </c>
       <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3366,6 +3533,7 @@
         </is>
       </c>
       <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3384,6 +3552,7 @@
         </is>
       </c>
       <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3402,6 +3571,7 @@
         </is>
       </c>
       <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3420,6 +3590,7 @@
         </is>
       </c>
       <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3438,6 +3609,7 @@
         </is>
       </c>
       <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3456,6 +3628,7 @@
         </is>
       </c>
       <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3474,6 +3647,7 @@
         </is>
       </c>
       <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3492,6 +3666,7 @@
         </is>
       </c>
       <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3510,6 +3685,7 @@
         </is>
       </c>
       <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3528,6 +3704,7 @@
         </is>
       </c>
       <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3546,6 +3723,7 @@
         </is>
       </c>
       <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3564,6 +3742,7 @@
         </is>
       </c>
       <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3582,6 +3761,7 @@
         </is>
       </c>
       <c r="D175" t="inlineStr"/>
+      <c r="E175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3600,6 +3780,7 @@
         </is>
       </c>
       <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3618,6 +3799,7 @@
         </is>
       </c>
       <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3636,6 +3818,7 @@
         </is>
       </c>
       <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3654,6 +3837,7 @@
         </is>
       </c>
       <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3672,6 +3856,7 @@
         </is>
       </c>
       <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3690,6 +3875,7 @@
         </is>
       </c>
       <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3708,6 +3894,7 @@
         </is>
       </c>
       <c r="D182" t="inlineStr"/>
+      <c r="E182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3726,6 +3913,7 @@
         </is>
       </c>
       <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3744,6 +3932,7 @@
         </is>
       </c>
       <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3762,6 +3951,7 @@
         </is>
       </c>
       <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3780,6 +3970,7 @@
         </is>
       </c>
       <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3798,6 +3989,7 @@
         </is>
       </c>
       <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3816,6 +4008,7 @@
         </is>
       </c>
       <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -3834,6 +4027,7 @@
         </is>
       </c>
       <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -3852,6 +4046,7 @@
         </is>
       </c>
       <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -3870,6 +4065,7 @@
         </is>
       </c>
       <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3888,6 +4084,7 @@
         </is>
       </c>
       <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -3906,6 +4103,7 @@
         </is>
       </c>
       <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -3924,6 +4122,7 @@
         </is>
       </c>
       <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -3942,6 +4141,7 @@
         </is>
       </c>
       <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3960,6 +4160,7 @@
         </is>
       </c>
       <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -3978,6 +4179,7 @@
         </is>
       </c>
       <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -3996,6 +4198,7 @@
         </is>
       </c>
       <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4014,6 +4217,7 @@
         </is>
       </c>
       <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4032,6 +4236,7 @@
         </is>
       </c>
       <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4050,6 +4255,7 @@
         </is>
       </c>
       <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4068,6 +4274,7 @@
         </is>
       </c>
       <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4086,6 +4293,7 @@
         </is>
       </c>
       <c r="D203" t="inlineStr"/>
+      <c r="E203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4104,6 +4312,7 @@
         </is>
       </c>
       <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4122,6 +4331,7 @@
         </is>
       </c>
       <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4140,6 +4350,7 @@
         </is>
       </c>
       <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4158,6 +4369,7 @@
         </is>
       </c>
       <c r="D207" t="inlineStr"/>
+      <c r="E207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4176,6 +4388,7 @@
         </is>
       </c>
       <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4194,6 +4407,7 @@
         </is>
       </c>
       <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -4212,6 +4426,7 @@
         </is>
       </c>
       <c r="D210" t="inlineStr"/>
+      <c r="E210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4230,6 +4445,7 @@
         </is>
       </c>
       <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -4248,6 +4464,7 @@
         </is>
       </c>
       <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -4266,6 +4483,7 @@
         </is>
       </c>
       <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -4284,6 +4502,7 @@
         </is>
       </c>
       <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -4302,6 +4521,7 @@
         </is>
       </c>
       <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -4320,6 +4540,7 @@
         </is>
       </c>
       <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -4338,6 +4559,7 @@
         </is>
       </c>
       <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -4356,6 +4578,7 @@
         </is>
       </c>
       <c r="D218" t="inlineStr"/>
+      <c r="E218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -4374,6 +4597,7 @@
         </is>
       </c>
       <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -4392,6 +4616,7 @@
         </is>
       </c>
       <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -4410,6 +4635,7 @@
         </is>
       </c>
       <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -4428,6 +4654,7 @@
         </is>
       </c>
       <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4446,6 +4673,7 @@
         </is>
       </c>
       <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -4464,6 +4692,7 @@
         </is>
       </c>
       <c r="D224" t="inlineStr"/>
+      <c r="E224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -4482,6 +4711,7 @@
         </is>
       </c>
       <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4500,6 +4730,7 @@
         </is>
       </c>
       <c r="D226" t="inlineStr"/>
+      <c r="E226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -4518,6 +4749,7 @@
         </is>
       </c>
       <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -4536,6 +4768,7 @@
         </is>
       </c>
       <c r="D228" t="inlineStr"/>
+      <c r="E228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4554,6 +4787,7 @@
         </is>
       </c>
       <c r="D229" t="inlineStr"/>
+      <c r="E229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4572,6 +4806,7 @@
         </is>
       </c>
       <c r="D230" t="inlineStr"/>
+      <c r="E230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -4590,6 +4825,7 @@
         </is>
       </c>
       <c r="D231" t="inlineStr"/>
+      <c r="E231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -4608,6 +4844,7 @@
         </is>
       </c>
       <c r="D232" t="inlineStr"/>
+      <c r="E232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4626,6 +4863,7 @@
         </is>
       </c>
       <c r="D233" t="inlineStr"/>
+      <c r="E233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -4644,6 +4882,7 @@
         </is>
       </c>
       <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4662,6 +4901,7 @@
         </is>
       </c>
       <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -4680,6 +4920,7 @@
         </is>
       </c>
       <c r="D236" t="inlineStr"/>
+      <c r="E236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -4698,6 +4939,7 @@
         </is>
       </c>
       <c r="D237" t="inlineStr"/>
+      <c r="E237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -4716,6 +4958,7 @@
         </is>
       </c>
       <c r="D238" t="inlineStr"/>
+      <c r="E238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -4734,6 +4977,7 @@
         </is>
       </c>
       <c r="D239" t="inlineStr"/>
+      <c r="E239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -4752,6 +4996,7 @@
         </is>
       </c>
       <c r="D240" t="inlineStr"/>
+      <c r="E240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -4770,6 +5015,7 @@
         </is>
       </c>
       <c r="D241" t="inlineStr"/>
+      <c r="E241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -4788,6 +5034,7 @@
         </is>
       </c>
       <c r="D242" t="inlineStr"/>
+      <c r="E242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -4806,6 +5053,7 @@
         </is>
       </c>
       <c r="D243" t="inlineStr"/>
+      <c r="E243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4824,6 +5072,7 @@
         </is>
       </c>
       <c r="D244" t="inlineStr"/>
+      <c r="E244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -4842,6 +5091,7 @@
         </is>
       </c>
       <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -4860,6 +5110,7 @@
         </is>
       </c>
       <c r="D246" t="inlineStr"/>
+      <c r="E246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -4878,6 +5129,7 @@
         </is>
       </c>
       <c r="D247" t="inlineStr"/>
+      <c r="E247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -4896,6 +5148,7 @@
         </is>
       </c>
       <c r="D248" t="inlineStr"/>
+      <c r="E248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -4914,6 +5167,7 @@
         </is>
       </c>
       <c r="D249" t="inlineStr"/>
+      <c r="E249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -4932,6 +5186,7 @@
         </is>
       </c>
       <c r="D250" t="inlineStr"/>
+      <c r="E250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -4950,6 +5205,7 @@
         </is>
       </c>
       <c r="D251" t="inlineStr"/>
+      <c r="E251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -4968,6 +5224,7 @@
         </is>
       </c>
       <c r="D252" t="inlineStr"/>
+      <c r="E252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -4986,6 +5243,7 @@
         </is>
       </c>
       <c r="D253" t="inlineStr"/>
+      <c r="E253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -5004,6 +5262,7 @@
         </is>
       </c>
       <c r="D254" t="inlineStr"/>
+      <c r="E254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -5022,6 +5281,7 @@
         </is>
       </c>
       <c r="D255" t="inlineStr"/>
+      <c r="E255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -5040,6 +5300,7 @@
         </is>
       </c>
       <c r="D256" t="inlineStr"/>
+      <c r="E256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -5058,6 +5319,7 @@
         </is>
       </c>
       <c r="D257" t="inlineStr"/>
+      <c r="E257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -5076,6 +5338,7 @@
         </is>
       </c>
       <c r="D258" t="inlineStr"/>
+      <c r="E258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -5094,6 +5357,7 @@
         </is>
       </c>
       <c r="D259" t="inlineStr"/>
+      <c r="E259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -5112,6 +5376,7 @@
         </is>
       </c>
       <c r="D260" t="inlineStr"/>
+      <c r="E260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -5130,6 +5395,7 @@
         </is>
       </c>
       <c r="D261" t="inlineStr"/>
+      <c r="E261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -5148,6 +5414,7 @@
         </is>
       </c>
       <c r="D262" t="inlineStr"/>
+      <c r="E262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -5166,6 +5433,7 @@
         </is>
       </c>
       <c r="D263" t="inlineStr"/>
+      <c r="E263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -5184,6 +5452,7 @@
         </is>
       </c>
       <c r="D264" t="inlineStr"/>
+      <c r="E264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -5202,6 +5471,7 @@
         </is>
       </c>
       <c r="D265" t="inlineStr"/>
+      <c r="E265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -5220,6 +5490,7 @@
         </is>
       </c>
       <c r="D266" t="inlineStr"/>
+      <c r="E266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -5238,6 +5509,7 @@
         </is>
       </c>
       <c r="D267" t="inlineStr"/>
+      <c r="E267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -5256,6 +5528,7 @@
         </is>
       </c>
       <c r="D268" t="inlineStr"/>
+      <c r="E268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -5274,6 +5547,7 @@
         </is>
       </c>
       <c r="D269" t="inlineStr"/>
+      <c r="E269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -5292,6 +5566,7 @@
         </is>
       </c>
       <c r="D270" t="inlineStr"/>
+      <c r="E270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -5310,6 +5585,7 @@
         </is>
       </c>
       <c r="D271" t="inlineStr"/>
+      <c r="E271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -5328,6 +5604,7 @@
         </is>
       </c>
       <c r="D272" t="inlineStr"/>
+      <c r="E272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -5346,6 +5623,7 @@
         </is>
       </c>
       <c r="D273" t="inlineStr"/>
+      <c r="E273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -5364,6 +5642,7 @@
         </is>
       </c>
       <c r="D274" t="inlineStr"/>
+      <c r="E274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -5382,6 +5661,7 @@
         </is>
       </c>
       <c r="D275" t="inlineStr"/>
+      <c r="E275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -5400,6 +5680,7 @@
         </is>
       </c>
       <c r="D276" t="inlineStr"/>
+      <c r="E276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -5418,6 +5699,7 @@
         </is>
       </c>
       <c r="D277" t="inlineStr"/>
+      <c r="E277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -5436,6 +5718,7 @@
         </is>
       </c>
       <c r="D278" t="inlineStr"/>
+      <c r="E278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -5454,6 +5737,7 @@
         </is>
       </c>
       <c r="D279" t="inlineStr"/>
+      <c r="E279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -5472,6 +5756,7 @@
         </is>
       </c>
       <c r="D280" t="inlineStr"/>
+      <c r="E280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -5490,6 +5775,7 @@
         </is>
       </c>
       <c r="D281" t="inlineStr"/>
+      <c r="E281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -5508,6 +5794,7 @@
         </is>
       </c>
       <c r="D282" t="inlineStr"/>
+      <c r="E282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -5526,6 +5813,7 @@
         </is>
       </c>
       <c r="D283" t="inlineStr"/>
+      <c r="E283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -5544,6 +5832,7 @@
         </is>
       </c>
       <c r="D284" t="inlineStr"/>
+      <c r="E284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -5562,6 +5851,7 @@
         </is>
       </c>
       <c r="D285" t="inlineStr"/>
+      <c r="E285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -5580,6 +5870,7 @@
         </is>
       </c>
       <c r="D286" t="inlineStr"/>
+      <c r="E286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -5598,6 +5889,7 @@
         </is>
       </c>
       <c r="D287" t="inlineStr"/>
+      <c r="E287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -5616,6 +5908,7 @@
         </is>
       </c>
       <c r="D288" t="inlineStr"/>
+      <c r="E288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -5634,6 +5927,7 @@
         </is>
       </c>
       <c r="D289" t="inlineStr"/>
+      <c r="E289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -5652,6 +5946,7 @@
         </is>
       </c>
       <c r="D290" t="inlineStr"/>
+      <c r="E290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -5670,6 +5965,7 @@
         </is>
       </c>
       <c r="D291" t="inlineStr"/>
+      <c r="E291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -5688,6 +5984,7 @@
         </is>
       </c>
       <c r="D292" t="inlineStr"/>
+      <c r="E292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -5706,6 +6003,7 @@
         </is>
       </c>
       <c r="D293" t="inlineStr"/>
+      <c r="E293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -5724,6 +6022,7 @@
         </is>
       </c>
       <c r="D294" t="inlineStr"/>
+      <c r="E294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -5742,6 +6041,7 @@
         </is>
       </c>
       <c r="D295" t="inlineStr"/>
+      <c r="E295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -5760,6 +6060,7 @@
         </is>
       </c>
       <c r="D296" t="inlineStr"/>
+      <c r="E296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -5778,6 +6079,7 @@
         </is>
       </c>
       <c r="D297" t="inlineStr"/>
+      <c r="E297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -5796,6 +6098,7 @@
         </is>
       </c>
       <c r="D298" t="inlineStr"/>
+      <c r="E298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -5814,6 +6117,7 @@
         </is>
       </c>
       <c r="D299" t="inlineStr"/>
+      <c r="E299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -5832,6 +6136,7 @@
         </is>
       </c>
       <c r="D300" t="inlineStr"/>
+      <c r="E300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -5850,6 +6155,7 @@
         </is>
       </c>
       <c r="D301" t="inlineStr"/>
+      <c r="E301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -5868,6 +6174,7 @@
         </is>
       </c>
       <c r="D302" t="inlineStr"/>
+      <c r="E302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -5886,6 +6193,7 @@
         </is>
       </c>
       <c r="D303" t="inlineStr"/>
+      <c r="E303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -5904,6 +6212,7 @@
         </is>
       </c>
       <c r="D304" t="inlineStr"/>
+      <c r="E304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -5922,6 +6231,7 @@
         </is>
       </c>
       <c r="D305" t="inlineStr"/>
+      <c r="E305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -5940,6 +6250,7 @@
         </is>
       </c>
       <c r="D306" t="inlineStr"/>
+      <c r="E306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -5958,6 +6269,7 @@
         </is>
       </c>
       <c r="D307" t="inlineStr"/>
+      <c r="E307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -5976,6 +6288,7 @@
         </is>
       </c>
       <c r="D308" t="inlineStr"/>
+      <c r="E308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -5994,6 +6307,7 @@
         </is>
       </c>
       <c r="D309" t="inlineStr"/>
+      <c r="E309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -6012,6 +6326,7 @@
         </is>
       </c>
       <c r="D310" t="inlineStr"/>
+      <c r="E310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -6030,6 +6345,7 @@
         </is>
       </c>
       <c r="D311" t="inlineStr"/>
+      <c r="E311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -6048,6 +6364,7 @@
         </is>
       </c>
       <c r="D312" t="inlineStr"/>
+      <c r="E312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -6066,6 +6383,7 @@
         </is>
       </c>
       <c r="D313" t="inlineStr"/>
+      <c r="E313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -6084,6 +6402,7 @@
         </is>
       </c>
       <c r="D314" t="inlineStr"/>
+      <c r="E314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -6102,6 +6421,7 @@
         </is>
       </c>
       <c r="D315" t="inlineStr"/>
+      <c r="E315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -6120,6 +6440,7 @@
         </is>
       </c>
       <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -6138,6 +6459,7 @@
         </is>
       </c>
       <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -6156,6 +6478,7 @@
         </is>
       </c>
       <c r="D318" t="inlineStr"/>
+      <c r="E318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -6174,6 +6497,7 @@
         </is>
       </c>
       <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -6192,6 +6516,7 @@
         </is>
       </c>
       <c r="D320" t="inlineStr"/>
+      <c r="E320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -6210,6 +6535,7 @@
         </is>
       </c>
       <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -6228,6 +6554,7 @@
         </is>
       </c>
       <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -6246,6 +6573,7 @@
         </is>
       </c>
       <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -6264,6 +6592,7 @@
         </is>
       </c>
       <c r="D324" t="inlineStr"/>
+      <c r="E324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -6282,6 +6611,7 @@
         </is>
       </c>
       <c r="D325" t="inlineStr"/>
+      <c r="E325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -6300,6 +6630,7 @@
         </is>
       </c>
       <c r="D326" t="inlineStr"/>
+      <c r="E326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -6318,6 +6649,7 @@
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
+      <c r="E327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -6336,6 +6668,7 @@
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
+      <c r="E328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -6354,6 +6687,7 @@
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -6372,6 +6706,7 @@
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
+      <c r="E330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -6390,6 +6725,7 @@
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
+      <c r="E331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -6408,6 +6744,7 @@
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
+      <c r="E332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -6426,6 +6763,7 @@
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
+      <c r="E333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -6444,6 +6782,7 @@
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
+      <c r="E334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -6462,6 +6801,7 @@
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
+      <c r="E335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -6480,6 +6820,7 @@
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -6498,6 +6839,7 @@
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
+      <c r="E337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -6516,6 +6858,7 @@
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
+      <c r="E338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -6534,6 +6877,7 @@
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -6552,6 +6896,7 @@
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -6570,6 +6915,7 @@
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
+      <c r="E341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -6588,6 +6934,7 @@
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
+      <c r="E342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -6606,6 +6953,7 @@
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
+      <c r="E343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -6624,6 +6972,7 @@
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
+      <c r="E344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -6642,6 +6991,7 @@
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -6660,6 +7010,7 @@
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -6678,6 +7029,7 @@
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
+      <c r="E347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -6696,6 +7048,7 @@
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
+      <c r="E348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -6714,6 +7067,7 @@
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
+      <c r="E349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -6732,6 +7086,7 @@
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
+      <c r="E350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -6750,6 +7105,7 @@
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
+      <c r="E351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -6768,6 +7124,7 @@
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
+      <c r="E352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -6786,6 +7143,7 @@
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
+      <c r="E353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -6804,6 +7162,7 @@
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
+      <c r="E354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -6822,6 +7181,7 @@
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
+      <c r="E355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -6840,6 +7200,7 @@
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
+      <c r="E356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -6858,6 +7219,7 @@
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
+      <c r="E357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -6876,6 +7238,7 @@
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
+      <c r="E358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -6894,6 +7257,7 @@
         </is>
       </c>
       <c r="D359" t="inlineStr"/>
+      <c r="E359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -6912,6 +7276,7 @@
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
+      <c r="E360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -6930,6 +7295,7 @@
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
+      <c r="E361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -6948,6 +7314,7 @@
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
+      <c r="E362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -6966,6 +7333,7 @@
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
+      <c r="E363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -6984,6 +7352,7 @@
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
+      <c r="E364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -7002,6 +7371,7 @@
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
+      <c r="E365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -7020,6 +7390,7 @@
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
+      <c r="E366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -7038,6 +7409,7 @@
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
+      <c r="E367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -7056,6 +7428,7 @@
         </is>
       </c>
       <c r="D368" t="inlineStr"/>
+      <c r="E368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -7074,6 +7447,7 @@
         </is>
       </c>
       <c r="D369" t="inlineStr"/>
+      <c r="E369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -7092,6 +7466,7 @@
         </is>
       </c>
       <c r="D370" t="inlineStr"/>
+      <c r="E370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -7110,6 +7485,7 @@
         </is>
       </c>
       <c r="D371" t="inlineStr"/>
+      <c r="E371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -7128,6 +7504,7 @@
         </is>
       </c>
       <c r="D372" t="inlineStr"/>
+      <c r="E372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -7146,6 +7523,7 @@
         </is>
       </c>
       <c r="D373" t="inlineStr"/>
+      <c r="E373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -7164,6 +7542,7 @@
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
+      <c r="E374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -7182,6 +7561,7 @@
         </is>
       </c>
       <c r="D375" t="inlineStr"/>
+      <c r="E375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -7200,6 +7580,7 @@
         </is>
       </c>
       <c r="D376" t="inlineStr"/>
+      <c r="E376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -7218,6 +7599,7 @@
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
+      <c r="E377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -7236,6 +7618,7 @@
         </is>
       </c>
       <c r="D378" t="inlineStr"/>
+      <c r="E378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -7254,6 +7637,7 @@
         </is>
       </c>
       <c r="D379" t="inlineStr"/>
+      <c r="E379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -7272,6 +7656,7 @@
         </is>
       </c>
       <c r="D380" t="inlineStr"/>
+      <c r="E380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -7290,6 +7675,7 @@
         </is>
       </c>
       <c r="D381" t="inlineStr"/>
+      <c r="E381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -7308,6 +7694,7 @@
         </is>
       </c>
       <c r="D382" t="inlineStr"/>
+      <c r="E382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -7326,6 +7713,7 @@
         </is>
       </c>
       <c r="D383" t="inlineStr"/>
+      <c r="E383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -7344,6 +7732,7 @@
         </is>
       </c>
       <c r="D384" t="inlineStr"/>
+      <c r="E384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -7362,6 +7751,7 @@
         </is>
       </c>
       <c r="D385" t="inlineStr"/>
+      <c r="E385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -7380,6 +7770,7 @@
         </is>
       </c>
       <c r="D386" t="inlineStr"/>
+      <c r="E386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -7398,6 +7789,7 @@
         </is>
       </c>
       <c r="D387" t="inlineStr"/>
+      <c r="E387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -7416,6 +7808,7 @@
         </is>
       </c>
       <c r="D388" t="inlineStr"/>
+      <c r="E388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -7434,6 +7827,7 @@
         </is>
       </c>
       <c r="D389" t="inlineStr"/>
+      <c r="E389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -7452,6 +7846,7 @@
         </is>
       </c>
       <c r="D390" t="inlineStr"/>
+      <c r="E390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -7470,6 +7865,7 @@
         </is>
       </c>
       <c r="D391" t="inlineStr"/>
+      <c r="E391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -7488,6 +7884,7 @@
         </is>
       </c>
       <c r="D392" t="inlineStr"/>
+      <c r="E392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -7506,6 +7903,7 @@
         </is>
       </c>
       <c r="D393" t="inlineStr"/>
+      <c r="E393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -7524,6 +7922,7 @@
         </is>
       </c>
       <c r="D394" t="inlineStr"/>
+      <c r="E394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -7542,6 +7941,7 @@
         </is>
       </c>
       <c r="D395" t="inlineStr"/>
+      <c r="E395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -7560,6 +7960,7 @@
         </is>
       </c>
       <c r="D396" t="inlineStr"/>
+      <c r="E396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -7578,6 +7979,7 @@
         </is>
       </c>
       <c r="D397" t="inlineStr"/>
+      <c r="E397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -7596,6 +7998,7 @@
         </is>
       </c>
       <c r="D398" t="inlineStr"/>
+      <c r="E398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -7614,6 +8017,7 @@
         </is>
       </c>
       <c r="D399" t="inlineStr"/>
+      <c r="E399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -7632,6 +8036,7 @@
         </is>
       </c>
       <c r="D400" t="inlineStr"/>
+      <c r="E400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -7650,6 +8055,7 @@
         </is>
       </c>
       <c r="D401" t="inlineStr"/>
+      <c r="E401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -7668,6 +8074,7 @@
         </is>
       </c>
       <c r="D402" t="inlineStr"/>
+      <c r="E402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -7686,6 +8093,7 @@
         </is>
       </c>
       <c r="D403" t="inlineStr"/>
+      <c r="E403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -7704,6 +8112,7 @@
         </is>
       </c>
       <c r="D404" t="inlineStr"/>
+      <c r="E404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -7722,6 +8131,7 @@
         </is>
       </c>
       <c r="D405" t="inlineStr"/>
+      <c r="E405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -7740,6 +8150,7 @@
         </is>
       </c>
       <c r="D406" t="inlineStr"/>
+      <c r="E406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -7758,6 +8169,7 @@
         </is>
       </c>
       <c r="D407" t="inlineStr"/>
+      <c r="E407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -7776,6 +8188,7 @@
         </is>
       </c>
       <c r="D408" t="inlineStr"/>
+      <c r="E408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -7794,11 +8207,15 @@
         </is>
       </c>
       <c r="D409" t="inlineStr"/>
+      <c r="E409" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="D2:D409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Reviewer A,Reviewer B"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implement reconciliation of human review decisions in screening steps
</commit_message>
<xml_diff>
--- a/data/review/gpt-5.4-pro/step-2-review.xlsx
+++ b/data/review/gpt-5.4-pro/step-2-review.xlsx
@@ -420,14 +420,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:F409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,12 +449,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>Review 1</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Reviewer</t>
+          <t>Review 2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Finale</t>
         </is>
       </c>
     </row>
@@ -475,6 +481,7 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -494,6 +501,7 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -513,6 +521,7 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -532,6 +541,7 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -551,6 +561,7 @@
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -570,6 +581,7 @@
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -589,6 +601,7 @@
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -608,6 +621,7 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -627,6 +641,7 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -646,6 +661,7 @@
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -665,6 +681,7 @@
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -684,6 +701,7 @@
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -703,6 +721,7 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -722,6 +741,7 @@
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -741,6 +761,7 @@
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -760,6 +781,7 @@
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -779,6 +801,7 @@
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -798,6 +821,7 @@
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -817,6 +841,7 @@
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -836,6 +861,7 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -855,6 +881,7 @@
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -874,6 +901,7 @@
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -893,6 +921,7 @@
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -912,6 +941,7 @@
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -931,6 +961,7 @@
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -950,6 +981,7 @@
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -969,6 +1001,7 @@
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -988,6 +1021,7 @@
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1007,6 +1041,7 @@
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1026,6 +1061,7 @@
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1045,6 +1081,7 @@
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1064,6 +1101,7 @@
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1083,6 +1121,7 @@
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1102,6 +1141,7 @@
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1121,6 +1161,7 @@
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1140,6 +1181,7 @@
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1159,6 +1201,7 @@
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1178,6 +1221,7 @@
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1197,6 +1241,7 @@
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1216,6 +1261,7 @@
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1235,6 +1281,7 @@
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1254,6 +1301,7 @@
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1273,6 +1321,7 @@
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1292,6 +1341,7 @@
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1311,6 +1361,7 @@
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1330,6 +1381,7 @@
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1349,6 +1401,7 @@
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1368,6 +1421,7 @@
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1387,6 +1441,7 @@
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1406,6 +1461,7 @@
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1425,6 +1481,7 @@
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1444,6 +1501,7 @@
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1463,6 +1521,7 @@
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1482,6 +1541,7 @@
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1501,6 +1561,7 @@
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1520,6 +1581,7 @@
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1539,6 +1601,7 @@
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1558,6 +1621,7 @@
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1577,6 +1641,7 @@
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1596,6 +1661,7 @@
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1615,6 +1681,7 @@
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1634,6 +1701,7 @@
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1653,6 +1721,7 @@
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1672,6 +1741,7 @@
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1691,6 +1761,7 @@
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1710,6 +1781,7 @@
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1729,6 +1801,7 @@
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1748,6 +1821,7 @@
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1767,6 +1841,7 @@
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1786,6 +1861,7 @@
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1805,6 +1881,7 @@
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1824,6 +1901,7 @@
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1843,6 +1921,7 @@
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1862,6 +1941,7 @@
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1881,6 +1961,7 @@
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1900,6 +1981,7 @@
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1919,6 +2001,7 @@
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1938,6 +2021,7 @@
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1957,6 +2041,7 @@
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1976,6 +2061,7 @@
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1995,6 +2081,7 @@
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2014,6 +2101,7 @@
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2033,6 +2121,7 @@
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2052,6 +2141,7 @@
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2071,6 +2161,7 @@
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2090,6 +2181,7 @@
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2109,6 +2201,7 @@
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2128,6 +2221,7 @@
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2147,6 +2241,7 @@
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2166,6 +2261,7 @@
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2185,6 +2281,7 @@
       </c>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2204,6 +2301,7 @@
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2223,6 +2321,7 @@
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2242,6 +2341,7 @@
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2261,6 +2361,7 @@
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2280,6 +2381,7 @@
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2299,6 +2401,7 @@
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2318,6 +2421,7 @@
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2337,6 +2441,7 @@
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2356,6 +2461,7 @@
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2375,6 +2481,7 @@
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2394,6 +2501,7 @@
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2413,6 +2521,7 @@
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2432,6 +2541,7 @@
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2451,6 +2561,7 @@
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2470,6 +2581,7 @@
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2489,6 +2601,7 @@
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2508,6 +2621,7 @@
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2527,6 +2641,7 @@
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2546,6 +2661,7 @@
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2565,6 +2681,7 @@
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2584,6 +2701,7 @@
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2603,6 +2721,7 @@
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2622,6 +2741,7 @@
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2641,6 +2761,7 @@
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2660,6 +2781,7 @@
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2679,6 +2801,7 @@
       </c>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2698,6 +2821,7 @@
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2717,6 +2841,7 @@
       </c>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2736,6 +2861,7 @@
       </c>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2755,6 +2881,7 @@
       </c>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2774,6 +2901,7 @@
       </c>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2793,6 +2921,7 @@
       </c>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2812,6 +2941,7 @@
       </c>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2831,6 +2961,7 @@
       </c>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2850,6 +2981,7 @@
       </c>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2869,6 +3001,7 @@
       </c>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2888,6 +3021,7 @@
       </c>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2907,6 +3041,7 @@
       </c>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2926,6 +3061,7 @@
       </c>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2945,6 +3081,7 @@
       </c>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2964,6 +3101,7 @@
       </c>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2983,6 +3121,7 @@
       </c>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3002,6 +3141,7 @@
       </c>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3021,6 +3161,7 @@
       </c>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3040,6 +3181,7 @@
       </c>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3059,6 +3201,7 @@
       </c>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3078,6 +3221,7 @@
       </c>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3097,6 +3241,7 @@
       </c>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3116,6 +3261,7 @@
       </c>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3135,6 +3281,7 @@
       </c>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3154,6 +3301,7 @@
       </c>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3173,6 +3321,7 @@
       </c>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3192,6 +3341,7 @@
       </c>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3211,6 +3361,7 @@
       </c>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3230,6 +3381,7 @@
       </c>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3249,6 +3401,7 @@
       </c>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3268,6 +3421,7 @@
       </c>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3287,6 +3441,7 @@
       </c>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3306,6 +3461,7 @@
       </c>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3325,6 +3481,7 @@
       </c>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3344,6 +3501,7 @@
       </c>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3363,6 +3521,7 @@
       </c>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3382,6 +3541,7 @@
       </c>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3401,6 +3561,7 @@
       </c>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3420,6 +3581,7 @@
       </c>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3439,6 +3601,7 @@
       </c>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3458,6 +3621,7 @@
       </c>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3477,6 +3641,7 @@
       </c>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3496,6 +3661,7 @@
       </c>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3515,6 +3681,7 @@
       </c>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3534,6 +3701,7 @@
       </c>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3553,6 +3721,7 @@
       </c>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3572,6 +3741,7 @@
       </c>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3591,6 +3761,7 @@
       </c>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3610,6 +3781,7 @@
       </c>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3629,6 +3801,7 @@
       </c>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3648,6 +3821,7 @@
       </c>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3667,6 +3841,7 @@
       </c>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3686,6 +3861,7 @@
       </c>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3705,6 +3881,7 @@
       </c>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3724,6 +3901,7 @@
       </c>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3743,6 +3921,7 @@
       </c>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3762,6 +3941,7 @@
       </c>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3781,6 +3961,7 @@
       </c>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3800,6 +3981,7 @@
       </c>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3819,6 +4001,7 @@
       </c>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3838,6 +4021,7 @@
       </c>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3857,6 +4041,7 @@
       </c>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3876,6 +4061,7 @@
       </c>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3895,6 +4081,7 @@
       </c>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3914,6 +4101,7 @@
       </c>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3933,6 +4121,7 @@
       </c>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3952,6 +4141,7 @@
       </c>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3971,6 +4161,7 @@
       </c>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3990,6 +4181,7 @@
       </c>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4009,6 +4201,7 @@
       </c>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4028,6 +4221,7 @@
       </c>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4047,6 +4241,7 @@
       </c>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4066,6 +4261,7 @@
       </c>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4085,6 +4281,7 @@
       </c>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4104,6 +4301,7 @@
       </c>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4123,6 +4321,7 @@
       </c>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4142,6 +4341,7 @@
       </c>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4161,6 +4361,7 @@
       </c>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4180,6 +4381,7 @@
       </c>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4199,6 +4401,7 @@
       </c>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4218,6 +4421,7 @@
       </c>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4237,6 +4441,7 @@
       </c>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4256,6 +4461,7 @@
       </c>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4275,6 +4481,7 @@
       </c>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4294,6 +4501,7 @@
       </c>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4313,6 +4521,7 @@
       </c>
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4332,6 +4541,7 @@
       </c>
       <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4351,6 +4561,7 @@
       </c>
       <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4370,6 +4581,7 @@
       </c>
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4389,6 +4601,7 @@
       </c>
       <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4408,6 +4621,7 @@
       </c>
       <c r="D209" t="inlineStr"/>
       <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -4427,6 +4641,7 @@
       </c>
       <c r="D210" t="inlineStr"/>
       <c r="E210" t="inlineStr"/>
+      <c r="F210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4446,6 +4661,7 @@
       </c>
       <c r="D211" t="inlineStr"/>
       <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -4465,6 +4681,7 @@
       </c>
       <c r="D212" t="inlineStr"/>
       <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -4484,6 +4701,7 @@
       </c>
       <c r="D213" t="inlineStr"/>
       <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -4503,6 +4721,7 @@
       </c>
       <c r="D214" t="inlineStr"/>
       <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -4522,6 +4741,7 @@
       </c>
       <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -4541,6 +4761,7 @@
       </c>
       <c r="D216" t="inlineStr"/>
       <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -4560,6 +4781,7 @@
       </c>
       <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -4579,6 +4801,7 @@
       </c>
       <c r="D218" t="inlineStr"/>
       <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -4598,6 +4821,7 @@
       </c>
       <c r="D219" t="inlineStr"/>
       <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -4617,6 +4841,7 @@
       </c>
       <c r="D220" t="inlineStr"/>
       <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -4636,6 +4861,7 @@
       </c>
       <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -4655,6 +4881,7 @@
       </c>
       <c r="D222" t="inlineStr"/>
       <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4674,6 +4901,7 @@
       </c>
       <c r="D223" t="inlineStr"/>
       <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -4693,6 +4921,7 @@
       </c>
       <c r="D224" t="inlineStr"/>
       <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -4712,6 +4941,7 @@
       </c>
       <c r="D225" t="inlineStr"/>
       <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4731,6 +4961,7 @@
       </c>
       <c r="D226" t="inlineStr"/>
       <c r="E226" t="inlineStr"/>
+      <c r="F226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -4750,6 +4981,7 @@
       </c>
       <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -4769,6 +5001,7 @@
       </c>
       <c r="D228" t="inlineStr"/>
       <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4788,6 +5021,7 @@
       </c>
       <c r="D229" t="inlineStr"/>
       <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4807,6 +5041,7 @@
       </c>
       <c r="D230" t="inlineStr"/>
       <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -4826,6 +5061,7 @@
       </c>
       <c r="D231" t="inlineStr"/>
       <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -4845,6 +5081,7 @@
       </c>
       <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4864,6 +5101,7 @@
       </c>
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -4883,6 +5121,7 @@
       </c>
       <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4902,6 +5141,7 @@
       </c>
       <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -4921,6 +5161,7 @@
       </c>
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -4940,6 +5181,7 @@
       </c>
       <c r="D237" t="inlineStr"/>
       <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -4959,6 +5201,7 @@
       </c>
       <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -4978,6 +5221,7 @@
       </c>
       <c r="D239" t="inlineStr"/>
       <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -4997,6 +5241,7 @@
       </c>
       <c r="D240" t="inlineStr"/>
       <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -5016,6 +5261,7 @@
       </c>
       <c r="D241" t="inlineStr"/>
       <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -5035,6 +5281,7 @@
       </c>
       <c r="D242" t="inlineStr"/>
       <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -5054,6 +5301,7 @@
       </c>
       <c r="D243" t="inlineStr"/>
       <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5073,6 +5321,7 @@
       </c>
       <c r="D244" t="inlineStr"/>
       <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5092,6 +5341,7 @@
       </c>
       <c r="D245" t="inlineStr"/>
       <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5111,6 +5361,7 @@
       </c>
       <c r="D246" t="inlineStr"/>
       <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5130,6 +5381,7 @@
       </c>
       <c r="D247" t="inlineStr"/>
       <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -5149,6 +5401,7 @@
       </c>
       <c r="D248" t="inlineStr"/>
       <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -5168,6 +5421,7 @@
       </c>
       <c r="D249" t="inlineStr"/>
       <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -5187,6 +5441,7 @@
       </c>
       <c r="D250" t="inlineStr"/>
       <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -5206,6 +5461,7 @@
       </c>
       <c r="D251" t="inlineStr"/>
       <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -5225,6 +5481,7 @@
       </c>
       <c r="D252" t="inlineStr"/>
       <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -5244,6 +5501,7 @@
       </c>
       <c r="D253" t="inlineStr"/>
       <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -5263,6 +5521,7 @@
       </c>
       <c r="D254" t="inlineStr"/>
       <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -5282,6 +5541,7 @@
       </c>
       <c r="D255" t="inlineStr"/>
       <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -5301,6 +5561,7 @@
       </c>
       <c r="D256" t="inlineStr"/>
       <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -5320,6 +5581,7 @@
       </c>
       <c r="D257" t="inlineStr"/>
       <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -5339,6 +5601,7 @@
       </c>
       <c r="D258" t="inlineStr"/>
       <c r="E258" t="inlineStr"/>
+      <c r="F258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -5358,6 +5621,7 @@
       </c>
       <c r="D259" t="inlineStr"/>
       <c r="E259" t="inlineStr"/>
+      <c r="F259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -5377,6 +5641,7 @@
       </c>
       <c r="D260" t="inlineStr"/>
       <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -5396,6 +5661,7 @@
       </c>
       <c r="D261" t="inlineStr"/>
       <c r="E261" t="inlineStr"/>
+      <c r="F261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -5415,6 +5681,7 @@
       </c>
       <c r="D262" t="inlineStr"/>
       <c r="E262" t="inlineStr"/>
+      <c r="F262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -5434,6 +5701,7 @@
       </c>
       <c r="D263" t="inlineStr"/>
       <c r="E263" t="inlineStr"/>
+      <c r="F263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -5453,6 +5721,7 @@
       </c>
       <c r="D264" t="inlineStr"/>
       <c r="E264" t="inlineStr"/>
+      <c r="F264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -5472,6 +5741,7 @@
       </c>
       <c r="D265" t="inlineStr"/>
       <c r="E265" t="inlineStr"/>
+      <c r="F265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -5491,6 +5761,7 @@
       </c>
       <c r="D266" t="inlineStr"/>
       <c r="E266" t="inlineStr"/>
+      <c r="F266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -5510,6 +5781,7 @@
       </c>
       <c r="D267" t="inlineStr"/>
       <c r="E267" t="inlineStr"/>
+      <c r="F267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -5529,6 +5801,7 @@
       </c>
       <c r="D268" t="inlineStr"/>
       <c r="E268" t="inlineStr"/>
+      <c r="F268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -5548,6 +5821,7 @@
       </c>
       <c r="D269" t="inlineStr"/>
       <c r="E269" t="inlineStr"/>
+      <c r="F269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -5567,6 +5841,7 @@
       </c>
       <c r="D270" t="inlineStr"/>
       <c r="E270" t="inlineStr"/>
+      <c r="F270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -5586,6 +5861,7 @@
       </c>
       <c r="D271" t="inlineStr"/>
       <c r="E271" t="inlineStr"/>
+      <c r="F271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -5605,6 +5881,7 @@
       </c>
       <c r="D272" t="inlineStr"/>
       <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -5624,6 +5901,7 @@
       </c>
       <c r="D273" t="inlineStr"/>
       <c r="E273" t="inlineStr"/>
+      <c r="F273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -5643,6 +5921,7 @@
       </c>
       <c r="D274" t="inlineStr"/>
       <c r="E274" t="inlineStr"/>
+      <c r="F274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -5662,6 +5941,7 @@
       </c>
       <c r="D275" t="inlineStr"/>
       <c r="E275" t="inlineStr"/>
+      <c r="F275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -5681,6 +5961,7 @@
       </c>
       <c r="D276" t="inlineStr"/>
       <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -5700,6 +5981,7 @@
       </c>
       <c r="D277" t="inlineStr"/>
       <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -5719,6 +6001,7 @@
       </c>
       <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr"/>
+      <c r="F278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -5738,6 +6021,7 @@
       </c>
       <c r="D279" t="inlineStr"/>
       <c r="E279" t="inlineStr"/>
+      <c r="F279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -5757,6 +6041,7 @@
       </c>
       <c r="D280" t="inlineStr"/>
       <c r="E280" t="inlineStr"/>
+      <c r="F280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -5776,6 +6061,7 @@
       </c>
       <c r="D281" t="inlineStr"/>
       <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -5795,6 +6081,7 @@
       </c>
       <c r="D282" t="inlineStr"/>
       <c r="E282" t="inlineStr"/>
+      <c r="F282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -5814,6 +6101,7 @@
       </c>
       <c r="D283" t="inlineStr"/>
       <c r="E283" t="inlineStr"/>
+      <c r="F283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -5833,6 +6121,7 @@
       </c>
       <c r="D284" t="inlineStr"/>
       <c r="E284" t="inlineStr"/>
+      <c r="F284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -5852,6 +6141,7 @@
       </c>
       <c r="D285" t="inlineStr"/>
       <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -5871,6 +6161,7 @@
       </c>
       <c r="D286" t="inlineStr"/>
       <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -5890,6 +6181,7 @@
       </c>
       <c r="D287" t="inlineStr"/>
       <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -5909,6 +6201,7 @@
       </c>
       <c r="D288" t="inlineStr"/>
       <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -5928,6 +6221,7 @@
       </c>
       <c r="D289" t="inlineStr"/>
       <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -5947,6 +6241,7 @@
       </c>
       <c r="D290" t="inlineStr"/>
       <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -5966,6 +6261,7 @@
       </c>
       <c r="D291" t="inlineStr"/>
       <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -5985,6 +6281,7 @@
       </c>
       <c r="D292" t="inlineStr"/>
       <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -6004,6 +6301,7 @@
       </c>
       <c r="D293" t="inlineStr"/>
       <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -6023,6 +6321,7 @@
       </c>
       <c r="D294" t="inlineStr"/>
       <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -6042,6 +6341,7 @@
       </c>
       <c r="D295" t="inlineStr"/>
       <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -6061,6 +6361,7 @@
       </c>
       <c r="D296" t="inlineStr"/>
       <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -6080,6 +6381,7 @@
       </c>
       <c r="D297" t="inlineStr"/>
       <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -6099,6 +6401,7 @@
       </c>
       <c r="D298" t="inlineStr"/>
       <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -6118,6 +6421,7 @@
       </c>
       <c r="D299" t="inlineStr"/>
       <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -6137,6 +6441,7 @@
       </c>
       <c r="D300" t="inlineStr"/>
       <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -6156,6 +6461,7 @@
       </c>
       <c r="D301" t="inlineStr"/>
       <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -6175,6 +6481,7 @@
       </c>
       <c r="D302" t="inlineStr"/>
       <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -6194,6 +6501,7 @@
       </c>
       <c r="D303" t="inlineStr"/>
       <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -6213,6 +6521,7 @@
       </c>
       <c r="D304" t="inlineStr"/>
       <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -6232,6 +6541,7 @@
       </c>
       <c r="D305" t="inlineStr"/>
       <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -6251,6 +6561,7 @@
       </c>
       <c r="D306" t="inlineStr"/>
       <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -6270,6 +6581,7 @@
       </c>
       <c r="D307" t="inlineStr"/>
       <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -6289,6 +6601,7 @@
       </c>
       <c r="D308" t="inlineStr"/>
       <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -6308,6 +6621,7 @@
       </c>
       <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr"/>
+      <c r="F309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -6327,6 +6641,7 @@
       </c>
       <c r="D310" t="inlineStr"/>
       <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -6346,6 +6661,7 @@
       </c>
       <c r="D311" t="inlineStr"/>
       <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -6365,6 +6681,7 @@
       </c>
       <c r="D312" t="inlineStr"/>
       <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -6384,6 +6701,7 @@
       </c>
       <c r="D313" t="inlineStr"/>
       <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -6403,6 +6721,7 @@
       </c>
       <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -6422,6 +6741,7 @@
       </c>
       <c r="D315" t="inlineStr"/>
       <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -6441,6 +6761,7 @@
       </c>
       <c r="D316" t="inlineStr"/>
       <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -6460,6 +6781,7 @@
       </c>
       <c r="D317" t="inlineStr"/>
       <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -6479,6 +6801,7 @@
       </c>
       <c r="D318" t="inlineStr"/>
       <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -6498,6 +6821,7 @@
       </c>
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -6517,6 +6841,7 @@
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr"/>
+      <c r="F320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -6536,6 +6861,7 @@
       </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -6555,6 +6881,7 @@
       </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -6574,6 +6901,7 @@
       </c>
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -6593,6 +6921,7 @@
       </c>
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr"/>
+      <c r="F324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -6612,6 +6941,7 @@
       </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr"/>
+      <c r="F325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -6631,6 +6961,7 @@
       </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -6650,6 +6981,7 @@
       </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -6669,6 +7001,7 @@
       </c>
       <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr"/>
+      <c r="F328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -6688,6 +7021,7 @@
       </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -6707,6 +7041,7 @@
       </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -6726,6 +7061,7 @@
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr"/>
+      <c r="F331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -6745,6 +7081,7 @@
       </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -6764,6 +7101,7 @@
       </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -6783,6 +7121,7 @@
       </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -6802,6 +7141,7 @@
       </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -6821,6 +7161,7 @@
       </c>
       <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr"/>
+      <c r="F336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -6840,6 +7181,7 @@
       </c>
       <c r="D337" t="inlineStr"/>
       <c r="E337" t="inlineStr"/>
+      <c r="F337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -6859,6 +7201,7 @@
       </c>
       <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr"/>
+      <c r="F338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -6878,6 +7221,7 @@
       </c>
       <c r="D339" t="inlineStr"/>
       <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -6897,6 +7241,7 @@
       </c>
       <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr"/>
+      <c r="F340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -6916,6 +7261,7 @@
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -6935,6 +7281,7 @@
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr"/>
+      <c r="F342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -6954,6 +7301,7 @@
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr"/>
+      <c r="F343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -6973,6 +7321,7 @@
       </c>
       <c r="D344" t="inlineStr"/>
       <c r="E344" t="inlineStr"/>
+      <c r="F344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -6992,6 +7341,7 @@
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr"/>
+      <c r="F345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -7011,6 +7361,7 @@
       </c>
       <c r="D346" t="inlineStr"/>
       <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -7030,6 +7381,7 @@
       </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -7049,6 +7401,7 @@
       </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -7068,6 +7421,7 @@
       </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -7087,6 +7441,7 @@
       </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -7106,6 +7461,7 @@
       </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -7125,6 +7481,7 @@
       </c>
       <c r="D352" t="inlineStr"/>
       <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -7144,6 +7501,7 @@
       </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -7163,6 +7521,7 @@
       </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -7182,6 +7541,7 @@
       </c>
       <c r="D355" t="inlineStr"/>
       <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -7201,6 +7561,7 @@
       </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -7220,6 +7581,7 @@
       </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -7239,6 +7601,7 @@
       </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -7258,6 +7621,7 @@
       </c>
       <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -7277,6 +7641,7 @@
       </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -7296,6 +7661,7 @@
       </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr"/>
+      <c r="F361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -7315,6 +7681,7 @@
       </c>
       <c r="D362" t="inlineStr"/>
       <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -7334,6 +7701,7 @@
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -7353,6 +7721,7 @@
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -7372,6 +7741,7 @@
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -7391,6 +7761,7 @@
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr"/>
+      <c r="F366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -7410,6 +7781,7 @@
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr"/>
+      <c r="F367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -7429,6 +7801,7 @@
       </c>
       <c r="D368" t="inlineStr"/>
       <c r="E368" t="inlineStr"/>
+      <c r="F368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -7448,6 +7821,7 @@
       </c>
       <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr"/>
+      <c r="F369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -7467,6 +7841,7 @@
       </c>
       <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr"/>
+      <c r="F370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -7486,6 +7861,7 @@
       </c>
       <c r="D371" t="inlineStr"/>
       <c r="E371" t="inlineStr"/>
+      <c r="F371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -7505,6 +7881,7 @@
       </c>
       <c r="D372" t="inlineStr"/>
       <c r="E372" t="inlineStr"/>
+      <c r="F372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -7524,6 +7901,7 @@
       </c>
       <c r="D373" t="inlineStr"/>
       <c r="E373" t="inlineStr"/>
+      <c r="F373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -7543,6 +7921,7 @@
       </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr"/>
+      <c r="F374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -7562,6 +7941,7 @@
       </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr"/>
+      <c r="F375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -7581,6 +7961,7 @@
       </c>
       <c r="D376" t="inlineStr"/>
       <c r="E376" t="inlineStr"/>
+      <c r="F376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -7600,6 +7981,7 @@
       </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr"/>
+      <c r="F377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -7619,6 +8001,7 @@
       </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr"/>
+      <c r="F378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -7638,6 +8021,7 @@
       </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr"/>
+      <c r="F379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -7657,6 +8041,7 @@
       </c>
       <c r="D380" t="inlineStr"/>
       <c r="E380" t="inlineStr"/>
+      <c r="F380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -7676,6 +8061,7 @@
       </c>
       <c r="D381" t="inlineStr"/>
       <c r="E381" t="inlineStr"/>
+      <c r="F381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -7695,6 +8081,7 @@
       </c>
       <c r="D382" t="inlineStr"/>
       <c r="E382" t="inlineStr"/>
+      <c r="F382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -7714,6 +8101,7 @@
       </c>
       <c r="D383" t="inlineStr"/>
       <c r="E383" t="inlineStr"/>
+      <c r="F383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -7733,6 +8121,7 @@
       </c>
       <c r="D384" t="inlineStr"/>
       <c r="E384" t="inlineStr"/>
+      <c r="F384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -7752,6 +8141,7 @@
       </c>
       <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr"/>
+      <c r="F385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -7771,6 +8161,7 @@
       </c>
       <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr"/>
+      <c r="F386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -7790,6 +8181,7 @@
       </c>
       <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr"/>
+      <c r="F387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -7809,6 +8201,7 @@
       </c>
       <c r="D388" t="inlineStr"/>
       <c r="E388" t="inlineStr"/>
+      <c r="F388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -7828,6 +8221,7 @@
       </c>
       <c r="D389" t="inlineStr"/>
       <c r="E389" t="inlineStr"/>
+      <c r="F389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -7847,6 +8241,7 @@
       </c>
       <c r="D390" t="inlineStr"/>
       <c r="E390" t="inlineStr"/>
+      <c r="F390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -7866,6 +8261,7 @@
       </c>
       <c r="D391" t="inlineStr"/>
       <c r="E391" t="inlineStr"/>
+      <c r="F391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -7885,6 +8281,7 @@
       </c>
       <c r="D392" t="inlineStr"/>
       <c r="E392" t="inlineStr"/>
+      <c r="F392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -7904,6 +8301,7 @@
       </c>
       <c r="D393" t="inlineStr"/>
       <c r="E393" t="inlineStr"/>
+      <c r="F393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -7923,6 +8321,7 @@
       </c>
       <c r="D394" t="inlineStr"/>
       <c r="E394" t="inlineStr"/>
+      <c r="F394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -7942,6 +8341,7 @@
       </c>
       <c r="D395" t="inlineStr"/>
       <c r="E395" t="inlineStr"/>
+      <c r="F395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -7961,6 +8361,7 @@
       </c>
       <c r="D396" t="inlineStr"/>
       <c r="E396" t="inlineStr"/>
+      <c r="F396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -7980,6 +8381,7 @@
       </c>
       <c r="D397" t="inlineStr"/>
       <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -7999,6 +8401,7 @@
       </c>
       <c r="D398" t="inlineStr"/>
       <c r="E398" t="inlineStr"/>
+      <c r="F398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -8018,6 +8421,7 @@
       </c>
       <c r="D399" t="inlineStr"/>
       <c r="E399" t="inlineStr"/>
+      <c r="F399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -8037,6 +8441,7 @@
       </c>
       <c r="D400" t="inlineStr"/>
       <c r="E400" t="inlineStr"/>
+      <c r="F400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -8056,6 +8461,7 @@
       </c>
       <c r="D401" t="inlineStr"/>
       <c r="E401" t="inlineStr"/>
+      <c r="F401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -8075,6 +8481,7 @@
       </c>
       <c r="D402" t="inlineStr"/>
       <c r="E402" t="inlineStr"/>
+      <c r="F402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -8094,6 +8501,7 @@
       </c>
       <c r="D403" t="inlineStr"/>
       <c r="E403" t="inlineStr"/>
+      <c r="F403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -8113,6 +8521,7 @@
       </c>
       <c r="D404" t="inlineStr"/>
       <c r="E404" t="inlineStr"/>
+      <c r="F404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -8132,6 +8541,7 @@
       </c>
       <c r="D405" t="inlineStr"/>
       <c r="E405" t="inlineStr"/>
+      <c r="F405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -8151,6 +8561,7 @@
       </c>
       <c r="D406" t="inlineStr"/>
       <c r="E406" t="inlineStr"/>
+      <c r="F406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -8170,6 +8581,7 @@
       </c>
       <c r="D407" t="inlineStr"/>
       <c r="E407" t="inlineStr"/>
+      <c r="F407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -8189,6 +8601,7 @@
       </c>
       <c r="D408" t="inlineStr"/>
       <c r="E408" t="inlineStr"/>
+      <c r="F408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -8208,14 +8621,18 @@
       </c>
       <c r="D409" t="inlineStr"/>
       <c r="E409" t="inlineStr"/>
+      <c r="F409" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="D2:D409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Reviewer A,Reviewer B"</formula1>
+      <formula1>"Include,Exclude"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>